<commit_message>
Fin Properties CG update
</commit_message>
<xml_diff>
--- a/Zephyr MK3/Data Files/ZephyrMK3_SimMasterFile.xlsx
+++ b/Zephyr MK3/Data Files/ZephyrMK3_SimMasterFile.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\grhfa\Desktop\Zephyr\Zephyr MK3\Data Files\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\grhfa\Desktop\Project-Zephyr\Zephyr MK3\Data Files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BAEEBBE1-1BE4-4EC5-8181-1FCBC771B48E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64ED9B62-4B8F-4B0B-9DD5-7FCCD0EACEBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -188,145 +188,145 @@
     <t>Fin Thickness</t>
   </si>
   <si>
+    <t>Leading Edge Distance from Nose Tip</t>
+  </si>
+  <si>
+    <t>lb/ft^3</t>
+  </si>
+  <si>
+    <t>Fin Density</t>
+  </si>
+  <si>
+    <t>Body Density</t>
+  </si>
+  <si>
+    <t>Nose Cone Length</t>
+  </si>
+  <si>
+    <t>Body Inner Diameter</t>
+  </si>
+  <si>
+    <t>Body Outer Diameter</t>
+  </si>
+  <si>
+    <t>Component Name</t>
+  </si>
+  <si>
+    <t>Deployment Bulkhead</t>
+  </si>
+  <si>
+    <t>Separation Bulkhead</t>
+  </si>
+  <si>
+    <t>Separation Coupler Tube</t>
+  </si>
+  <si>
+    <t>Distance from Nose Tip (in)</t>
+  </si>
+  <si>
+    <t>Dart Drogue Chute</t>
+  </si>
+  <si>
+    <t>Symbol</t>
+  </si>
+  <si>
+    <t>gamma</t>
+  </si>
+  <si>
+    <t>R</t>
+  </si>
+  <si>
+    <t>p_atm</t>
+  </si>
+  <si>
+    <t>T_atm</t>
+  </si>
+  <si>
+    <t>mach_min</t>
+  </si>
+  <si>
+    <t>mach_max</t>
+  </si>
+  <si>
+    <t>mach_inc</t>
+  </si>
+  <si>
+    <t>alpha_min</t>
+  </si>
+  <si>
+    <t>alpha_max</t>
+  </si>
+  <si>
+    <t>alpha_inc</t>
+  </si>
+  <si>
+    <t>bodyOuterDiameter</t>
+  </si>
+  <si>
+    <t>bodyInnerDiameter</t>
+  </si>
+  <si>
+    <t>noseLength</t>
+  </si>
+  <si>
+    <t>bodyDensity</t>
+  </si>
+  <si>
+    <t>finDensity</t>
+  </si>
+  <si>
+    <t>finRes</t>
+  </si>
+  <si>
+    <t>numStages</t>
+  </si>
+  <si>
+    <t>numFins</t>
+  </si>
+  <si>
+    <t>rootChord</t>
+  </si>
+  <si>
+    <t>tipChord</t>
+  </si>
+  <si>
+    <t>height</t>
+  </si>
+  <si>
+    <t>sweepLength</t>
+  </si>
+  <si>
+    <t>thickness</t>
+  </si>
+  <si>
+    <t>leadDistance</t>
+  </si>
+  <si>
+    <t>Trailing Edge Distance from Stage End</t>
+  </si>
+  <si>
+    <t>trailDistance</t>
+  </si>
+  <si>
+    <t>Surface Gravity</t>
+  </si>
+  <si>
+    <t>ft/s^2</t>
+  </si>
+  <si>
+    <t>g0</t>
+  </si>
+  <si>
     <t>Leading Edge Taper Length</t>
   </si>
   <si>
     <t>Trailing Edge Taper Length</t>
   </si>
   <si>
-    <t>Leading Edge Distance from Nose Tip</t>
-  </si>
-  <si>
-    <t>lb/ft^3</t>
-  </si>
-  <si>
-    <t>Fin Density</t>
-  </si>
-  <si>
-    <t>Body Density</t>
-  </si>
-  <si>
-    <t>Nose Cone Length</t>
-  </si>
-  <si>
-    <t>Body Inner Diameter</t>
-  </si>
-  <si>
-    <t>Body Outer Diameter</t>
-  </si>
-  <si>
-    <t>Component Name</t>
-  </si>
-  <si>
-    <t>Deployment Bulkhead</t>
-  </si>
-  <si>
-    <t>Separation Bulkhead</t>
-  </si>
-  <si>
-    <t>Separation Coupler Tube</t>
-  </si>
-  <si>
-    <t>Distance from Nose Tip (in)</t>
-  </si>
-  <si>
-    <t>Dart Drogue Chute</t>
-  </si>
-  <si>
-    <t>Symbol</t>
-  </si>
-  <si>
-    <t>gamma</t>
-  </si>
-  <si>
-    <t>R</t>
-  </si>
-  <si>
-    <t>p_atm</t>
-  </si>
-  <si>
-    <t>T_atm</t>
-  </si>
-  <si>
-    <t>mach_min</t>
-  </si>
-  <si>
-    <t>mach_max</t>
-  </si>
-  <si>
-    <t>mach_inc</t>
-  </si>
-  <si>
-    <t>alpha_min</t>
-  </si>
-  <si>
-    <t>alpha_max</t>
-  </si>
-  <si>
-    <t>alpha_inc</t>
-  </si>
-  <si>
-    <t>bodyOuterDiameter</t>
-  </si>
-  <si>
-    <t>bodyInnerDiameter</t>
-  </si>
-  <si>
-    <t>noseLength</t>
-  </si>
-  <si>
-    <t>bodyDensity</t>
-  </si>
-  <si>
-    <t>finDensity</t>
-  </si>
-  <si>
-    <t>finRes</t>
-  </si>
-  <si>
-    <t>numStages</t>
-  </si>
-  <si>
-    <t>numFins</t>
-  </si>
-  <si>
-    <t>rootChord</t>
-  </si>
-  <si>
-    <t>tipChord</t>
-  </si>
-  <si>
-    <t>height</t>
-  </si>
-  <si>
-    <t>sweepLength</t>
-  </si>
-  <si>
-    <t>thickness</t>
-  </si>
-  <si>
     <t>leadTaperLength</t>
   </si>
   <si>
     <t>trailTaperLength</t>
-  </si>
-  <si>
-    <t>leadDistance</t>
-  </si>
-  <si>
-    <t>Trailing Edge Distance from Stage End</t>
-  </si>
-  <si>
-    <t>trailDistance</t>
-  </si>
-  <si>
-    <t>Surface Gravity</t>
-  </si>
-  <si>
-    <t>ft/s^2</t>
-  </si>
-  <si>
-    <t>g0</t>
   </si>
 </sst>
 </file>
@@ -882,7 +882,7 @@
     <col min="8" max="8" width="7.5546875" style="5" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="32.5546875" style="12" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="5.44140625" style="15" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="15.21875" style="15" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="18.77734375" style="15" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="8.109375" style="15" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="8.109375" style="5" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="22.21875" style="12" bestFit="1" customWidth="1"/>
@@ -929,7 +929,7 @@
         <v>42</v>
       </c>
       <c r="C2" s="10" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="D2" s="11" t="s">
         <v>43</v>
@@ -941,7 +941,7 @@
         <v>42</v>
       </c>
       <c r="G2" s="10" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="H2" s="11" t="s">
         <v>43</v>
@@ -953,7 +953,7 @@
         <v>44</v>
       </c>
       <c r="K2" s="10" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="L2" s="10" t="s">
         <v>3</v>
@@ -962,7 +962,7 @@
         <v>4</v>
       </c>
       <c r="N2" s="22" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="O2" s="10" t="s">
         <v>24</v>
@@ -971,7 +971,7 @@
         <v>25</v>
       </c>
       <c r="Q2" s="27" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
     <row r="3" spans="1:19" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
@@ -982,19 +982,19 @@
         <v>1</v>
       </c>
       <c r="C3" s="15" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="D3" s="5">
         <v>1.4</v>
       </c>
       <c r="E3" s="18" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="F3" s="21" t="s">
         <v>26</v>
       </c>
       <c r="G3" s="21" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="H3" s="6">
         <v>3.12</v>
@@ -1006,7 +1006,7 @@
         <v>1</v>
       </c>
       <c r="K3" s="17" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="L3" s="24">
         <v>4</v>
@@ -1035,19 +1035,19 @@
         <v>29</v>
       </c>
       <c r="C4" s="15" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="D4" s="5">
         <v>1716</v>
       </c>
       <c r="E4" s="13" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="F4" s="16" t="s">
         <v>26</v>
       </c>
       <c r="G4" s="29" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H4" s="5">
         <v>3</v>
@@ -1059,7 +1059,7 @@
         <v>26</v>
       </c>
       <c r="K4" s="21" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="L4" s="25">
         <v>4.6879999999999997</v>
@@ -1082,25 +1082,25 @@
     </row>
     <row r="5" spans="1:19" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="12" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="B5" s="15" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="C5" s="15" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="D5" s="5">
         <v>32.173999999999999</v>
       </c>
       <c r="E5" s="18" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="F5" s="21" t="s">
         <v>26</v>
       </c>
       <c r="G5" s="21" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="H5" s="6">
         <v>15</v>
@@ -1112,7 +1112,7 @@
         <v>26</v>
       </c>
       <c r="K5" s="21" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="L5" s="25">
         <v>2.375</v>
@@ -1141,19 +1141,19 @@
         <v>28</v>
       </c>
       <c r="C6" s="15" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="D6" s="5">
         <v>14.696</v>
       </c>
       <c r="E6" s="18" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="F6" s="17" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="G6" s="21" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="H6" s="5">
         <v>124</v>
@@ -1165,7 +1165,7 @@
         <v>26</v>
       </c>
       <c r="K6" s="21" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="L6" s="25">
         <v>2.6019999999999999</v>
@@ -1195,19 +1195,19 @@
         <v>30</v>
       </c>
       <c r="C7" s="29" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D7" s="5">
         <v>59</v>
       </c>
       <c r="E7" s="19" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="F7" s="17" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="G7" s="21" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="H7" s="6">
         <v>83.8</v>
@@ -1219,7 +1219,7 @@
         <v>26</v>
       </c>
       <c r="K7" s="21" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="L7" s="25">
         <v>2.3130000000000002</v>
@@ -1248,7 +1248,7 @@
         <v>31</v>
       </c>
       <c r="C8" s="17" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="D8" s="6">
         <v>0</v>
@@ -1263,7 +1263,7 @@
         <v>26</v>
       </c>
       <c r="K8" s="21" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="L8" s="26">
         <v>0.25</v>
@@ -1272,7 +1272,7 @@
         <v>0.25</v>
       </c>
       <c r="N8" s="18" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="O8" s="17">
         <v>1.7999999999999999E-2</v>
@@ -1292,7 +1292,7 @@
         <v>31</v>
       </c>
       <c r="C9" s="17" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="D9" s="6">
         <v>2</v>
@@ -1301,13 +1301,13 @@
       <c r="F9" s="21"/>
       <c r="G9" s="21"/>
       <c r="I9" s="18" t="s">
-        <v>50</v>
+        <v>93</v>
       </c>
       <c r="J9" s="17" t="s">
         <v>26</v>
       </c>
       <c r="K9" s="21" t="s">
-        <v>89</v>
+        <v>95</v>
       </c>
       <c r="L9" s="24">
         <v>0</v>
@@ -1336,19 +1336,19 @@
         <v>31</v>
       </c>
       <c r="C10" s="17" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="D10" s="6">
         <v>0.01</v>
       </c>
-      <c r="I10" s="18" t="s">
-        <v>51</v>
-      </c>
-      <c r="J10" s="17" t="s">
+      <c r="I10" s="12" t="s">
+        <v>94</v>
+      </c>
+      <c r="J10" s="15" t="s">
         <v>26</v>
       </c>
       <c r="K10" s="21" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="L10" s="24">
         <v>0</v>
@@ -1357,7 +1357,7 @@
         <v>0</v>
       </c>
       <c r="N10" s="13" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="O10" s="15">
         <v>0.193</v>
@@ -1377,19 +1377,19 @@
         <v>32</v>
       </c>
       <c r="C11" s="17" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="D11" s="6">
         <v>0</v>
       </c>
       <c r="I11" s="18" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="J11" s="17" t="s">
         <v>26</v>
       </c>
       <c r="K11" s="21" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="L11" s="24">
         <v>48.3</v>
@@ -1418,19 +1418,19 @@
         <v>32</v>
       </c>
       <c r="C12" s="17" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="D12" s="6">
         <v>5</v>
       </c>
       <c r="I12" s="12" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="J12" s="15" t="s">
         <v>26</v>
       </c>
       <c r="K12" s="15" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="L12" s="15">
         <v>0</v>
@@ -1460,16 +1460,11 @@
         <v>32</v>
       </c>
       <c r="C13" s="17" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="D13" s="6">
         <v>0.1</v>
       </c>
-      <c r="I13" s="14"/>
-      <c r="J13" s="17"/>
-      <c r="K13" s="17"/>
-      <c r="L13" s="24"/>
-      <c r="M13" s="7"/>
       <c r="N13" s="18" t="s">
         <v>14</v>
       </c>
@@ -1491,18 +1486,13 @@
         <v>1</v>
       </c>
       <c r="C14" s="17" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="D14" s="6">
         <v>100</v>
       </c>
-      <c r="I14" s="14"/>
-      <c r="J14" s="17"/>
-      <c r="K14" s="17"/>
-      <c r="L14" s="24"/>
-      <c r="M14" s="7"/>
       <c r="N14" s="13" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="O14" s="17">
         <v>0.16300000000000001</v>
@@ -1522,13 +1512,13 @@
         <v>1</v>
       </c>
       <c r="C15" s="17" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="D15" s="6">
         <v>2</v>
       </c>
       <c r="N15" s="18" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="O15" s="17">
         <v>0.308</v>

</xml_diff>

<commit_message>
Updated CG to account for manufacturability
</commit_message>
<xml_diff>
--- a/Zephyr MK3/Data Files/ZephyrMK3_SimMasterFile.xlsx
+++ b/Zephyr MK3/Data Files/ZephyrMK3_SimMasterFile.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\grhfa\Desktop\Project-Zephyr\Zephyr MK3\Data Files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64ED9B62-4B8F-4B0B-9DD5-7FCCD0EACEBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F71205D4-BD6B-4B7E-BD56-D0718FCB90FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="101">
   <si>
     <t>Setup</t>
   </si>
@@ -327,6 +327,18 @@
   </si>
   <si>
     <t>trailTaperLength</t>
+  </si>
+  <si>
+    <t>Leading Edge Thickness</t>
+  </si>
+  <si>
+    <t>leadThickness</t>
+  </si>
+  <si>
+    <t>Trailing Edge Thickness</t>
+  </si>
+  <si>
+    <t>trailThickness</t>
   </si>
 </sst>
 </file>
@@ -1342,18 +1354,18 @@
         <v>0.01</v>
       </c>
       <c r="I10" s="12" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="J10" s="15" t="s">
         <v>26</v>
       </c>
-      <c r="K10" s="21" t="s">
-        <v>96</v>
-      </c>
-      <c r="L10" s="24">
+      <c r="K10" s="15" t="s">
+        <v>98</v>
+      </c>
+      <c r="L10" s="15">
         <v>0</v>
       </c>
-      <c r="M10" s="7">
+      <c r="M10" s="5">
         <v>0</v>
       </c>
       <c r="N10" s="13" t="s">
@@ -1424,18 +1436,18 @@
         <v>5</v>
       </c>
       <c r="I12" s="12" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="J12" s="15" t="s">
         <v>26</v>
       </c>
-      <c r="K12" s="15" t="s">
-        <v>89</v>
-      </c>
-      <c r="L12" s="15">
+      <c r="K12" s="21" t="s">
+        <v>96</v>
+      </c>
+      <c r="L12" s="24">
         <v>0</v>
       </c>
-      <c r="M12" s="5">
+      <c r="M12" s="7">
         <v>0</v>
       </c>
       <c r="N12" s="14" t="s">
@@ -1465,6 +1477,21 @@
       <c r="D13" s="6">
         <v>0.1</v>
       </c>
+      <c r="I13" s="12" t="s">
+        <v>99</v>
+      </c>
+      <c r="J13" s="15" t="s">
+        <v>26</v>
+      </c>
+      <c r="K13" s="15" t="s">
+        <v>100</v>
+      </c>
+      <c r="L13" s="15">
+        <v>0</v>
+      </c>
+      <c r="M13" s="5">
+        <v>0</v>
+      </c>
       <c r="N13" s="18" t="s">
         <v>14</v>
       </c>
@@ -1490,6 +1517,21 @@
       </c>
       <c r="D14" s="6">
         <v>100</v>
+      </c>
+      <c r="I14" s="12" t="s">
+        <v>88</v>
+      </c>
+      <c r="J14" s="15" t="s">
+        <v>26</v>
+      </c>
+      <c r="K14" s="15" t="s">
+        <v>89</v>
+      </c>
+      <c r="L14" s="15">
+        <v>0</v>
+      </c>
+      <c r="M14" s="5">
+        <v>0</v>
       </c>
       <c r="N14" s="13" t="s">
         <v>59</v>

</xml_diff>